<commit_message>
ftp-app-8.0.2.019 added skip row criteria in ndTo1d
</commit_message>
<xml_diff>
--- a/FTP/meta-data/test-data/nd-to-1d-data/nd-to-1d-data.xlsx
+++ b/FTP/meta-data/test-data/nd-to-1d-data/nd-to-1d-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\ftp-application\FTP\meta-data\test-data\nd-to-1d-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1C41A60-5506-42C3-A951-4ACA4CD4598D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE3ECD72-6A9D-4BF7-AF72-2E79F50EEF1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{16FE5A34-0522-4997-AF06-71F88BC9C3ED}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{16FE5A34-0522-4997-AF06-71F88BC9C3ED}"/>
   </bookViews>
   <sheets>
     <sheet name="2d" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="47">
   <si>
     <t>SN</t>
   </si>
@@ -160,6 +160,24 @@
   </si>
   <si>
     <t>R</t>
+  </si>
+  <si>
+    <t>XYZ</t>
+  </si>
+  <si>
+    <t>BR</t>
+  </si>
+  <si>
+    <t>PQR</t>
+  </si>
+  <si>
+    <t>BR2</t>
+  </si>
+  <si>
+    <t>UP2</t>
+  </si>
+  <si>
+    <t>ABC</t>
   </si>
 </sst>
 </file>
@@ -617,7 +635,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE6CBDE8-0EA7-48DD-8512-3542567C08AA}">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="11.6640625" customWidth="1"/>
@@ -781,6 +799,45 @@
       </c>
       <c r="H6" t="s">
         <v>19</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" s="1">
+        <v>5</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="C7" t="s">
+        <v>42</v>
+      </c>
+      <c r="G7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" s="1">
+        <v>6</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="D8" t="s">
+        <v>44</v>
+      </c>
+      <c r="G8" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" s="1">
+        <v>7</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
ftp-app-8.0.2.019 test case improved for nd to 1d
</commit_message>
<xml_diff>
--- a/FTP/meta-data/test-data/nd-to-1d-data/nd-to-1d-data.xlsx
+++ b/FTP/meta-data/test-data/nd-to-1d-data/nd-to-1d-data.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\ftp-application\FTP\meta-data\test-data\nd-to-1d-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE3ECD72-6A9D-4BF7-AF72-2E79F50EEF1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9519427D-DEEE-4772-A968-B84377826DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{16FE5A34-0522-4997-AF06-71F88BC9C3ED}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{16FE5A34-0522-4997-AF06-71F88BC9C3ED}"/>
   </bookViews>
   <sheets>
     <sheet name="2d" sheetId="1" r:id="rId1"/>
     <sheet name="3d" sheetId="2" r:id="rId2"/>
-    <sheet name="2d_1" sheetId="3" r:id="rId3"/>
-    <sheet name="1d" sheetId="4" r:id="rId4"/>
+    <sheet name="3d_1" sheetId="5" r:id="rId3"/>
+    <sheet name="2d_1" sheetId="3" r:id="rId4"/>
+    <sheet name="1d" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="65">
   <si>
     <t>SN</t>
   </si>
@@ -178,6 +179,60 @@
   </si>
   <si>
     <t>ABC</t>
+  </si>
+  <si>
+    <t>R1</t>
+  </si>
+  <si>
+    <t>Location</t>
+  </si>
+  <si>
+    <t>Row no</t>
+  </si>
+  <si>
+    <t>WG</t>
+  </si>
+  <si>
+    <t>R2</t>
+  </si>
+  <si>
+    <t>R3</t>
+  </si>
+  <si>
+    <t>17 HR</t>
+  </si>
+  <si>
+    <t>C17 HR</t>
+  </si>
+  <si>
+    <t>SH19 HR</t>
+  </si>
+  <si>
+    <t>C21 HR</t>
+  </si>
+  <si>
+    <t>29 HR</t>
+  </si>
+  <si>
+    <t>SH27 HR</t>
+  </si>
+  <si>
+    <t>23 HR</t>
+  </si>
+  <si>
+    <t>13 DR</t>
+  </si>
+  <si>
+    <t>DD(LAD) HHR</t>
+  </si>
+  <si>
+    <t>DD (HTE) DR</t>
+  </si>
+  <si>
+    <t>2 HR</t>
+  </si>
+  <si>
+    <t>2EUR</t>
   </si>
 </sst>
 </file>
@@ -213,7 +268,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -223,6 +278,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -851,6 +909,118 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8D100159-999C-47DD-8475-273C50AEEF64}">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="15.5546875" customWidth="1"/>
+    <col min="4" max="4" width="14.77734375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C1" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="4">
+        <v>1</v>
+      </c>
+      <c r="D2" s="4">
+        <v>2</v>
+      </c>
+      <c r="E2" s="4">
+        <v>1</v>
+      </c>
+      <c r="F2" s="4">
+        <v>2</v>
+      </c>
+      <c r="G2" s="4">
+        <v>1</v>
+      </c>
+      <c r="H2" s="4">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>50</v>
+      </c>
+      <c r="B3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" t="s">
+        <v>62</v>
+      </c>
+      <c r="E3" t="s">
+        <v>57</v>
+      </c>
+      <c r="F3" t="s">
+        <v>58</v>
+      </c>
+      <c r="G3" t="s">
+        <v>53</v>
+      </c>
+      <c r="H3" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>50</v>
+      </c>
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E4" t="s">
+        <v>59</v>
+      </c>
+      <c r="F4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G4" t="s">
+        <v>55</v>
+      </c>
+      <c r="H4" t="s">
+        <v>56</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7FC4263-E33F-4DFE-9240-DD92FC1E7EF6}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -932,7 +1102,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29401365-B411-4B64-80A1-27BF962D067F}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>

<commit_message>
ftp-app-8.0.2.019 data dimention config parameter removed from ndto1d config
</commit_message>
<xml_diff>
--- a/FTP/meta-data/test-data/nd-to-1d-data/nd-to-1d-data.xlsx
+++ b/FTP/meta-data/test-data/nd-to-1d-data/nd-to-1d-data.xlsx
@@ -1,23 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\ftp-application\FTP\meta-data\test-data\nd-to-1d-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9519427D-DEEE-4772-A968-B84377826DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2F2989B-E598-4CBD-A771-D17DF9E2E444}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{16FE5A34-0522-4997-AF06-71F88BC9C3ED}"/>
+    <workbookView xWindow="5760" yWindow="3360" windowWidth="17280" windowHeight="8880" activeTab="3" xr2:uid="{16FE5A34-0522-4997-AF06-71F88BC9C3ED}"/>
   </bookViews>
   <sheets>
     <sheet name="2d" sheetId="1" r:id="rId1"/>
     <sheet name="3d" sheetId="2" r:id="rId2"/>
     <sheet name="3d_1" sheetId="5" r:id="rId3"/>
-    <sheet name="2d_1" sheetId="3" r:id="rId4"/>
-    <sheet name="1d" sheetId="4" r:id="rId5"/>
+    <sheet name="3d_2" sheetId="6" r:id="rId4"/>
+    <sheet name="3d_2_expected" sheetId="7" r:id="rId5"/>
+    <sheet name="2d_1" sheetId="3" r:id="rId6"/>
+    <sheet name="1d" sheetId="4" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="86">
   <si>
     <t>SN</t>
   </si>
@@ -233,6 +235,69 @@
   </si>
   <si>
     <t>2EUR</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>ID-1</t>
+  </si>
+  <si>
+    <t>ID-2</t>
+  </si>
+  <si>
+    <t>V5 val para-1</t>
+  </si>
+  <si>
+    <t>V4 val para-1</t>
+  </si>
+  <si>
+    <t>Para-1 matching</t>
+  </si>
+  <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>y</t>
+  </si>
+  <si>
+    <t>No</t>
+  </si>
+  <si>
+    <t>p</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>V5 val para-2</t>
+  </si>
+  <si>
+    <t>V4 val para-2</t>
+  </si>
+  <si>
+    <t>Para-2 matching</t>
+  </si>
+  <si>
+    <t>Para-2</t>
+  </si>
+  <si>
+    <t>Para-1</t>
+  </si>
+  <si>
+    <t>p1</t>
+  </si>
+  <si>
+    <t>p3</t>
+  </si>
+  <si>
+    <t>p4</t>
+  </si>
+  <si>
+    <t>X</t>
+  </si>
+  <si>
+    <t>Y</t>
   </si>
 </sst>
 </file>
@@ -277,10 +342,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -707,18 +772,18 @@
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3" t="s">
+      <c r="D1" s="4"/>
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3" t="s">
+      <c r="F1" s="4"/>
+      <c r="G1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="3"/>
+      <c r="H1" s="4"/>
       <c r="I1" s="2" t="s">
         <v>2</v>
       </c>
@@ -917,49 +982,49 @@
     <col min="4" max="4" width="14.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="C1" s="4" t="s">
+    <row r="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="C1" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="G1" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="2" spans="1:8" s="4" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="C2" s="4">
+      <c r="C2" s="3">
         <v>1</v>
       </c>
-      <c r="D2" s="4">
+      <c r="D2" s="3">
         <v>2</v>
       </c>
-      <c r="E2" s="4">
+      <c r="E2" s="3">
         <v>1</v>
       </c>
-      <c r="F2" s="4">
+      <c r="F2" s="3">
         <v>2</v>
       </c>
-      <c r="G2" s="4">
+      <c r="G2" s="3">
         <v>1</v>
       </c>
-      <c r="H2" s="4">
+      <c r="H2" s="3">
         <v>2</v>
       </c>
     </row>
@@ -1021,6 +1086,179 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A67E543-EE22-4B92-ADC8-8D559B12F1D9}">
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E2" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>77</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>66</v>
+      </c>
+      <c r="B4" t="s">
+        <v>71</v>
+      </c>
+      <c r="C4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E4" t="s">
+        <v>81</v>
+      </c>
+      <c r="F4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B5" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" t="s">
+        <v>74</v>
+      </c>
+      <c r="D5" t="s">
+        <v>75</v>
+      </c>
+      <c r="E5" t="s">
+        <v>82</v>
+      </c>
+      <c r="F5" t="s">
+        <v>83</v>
+      </c>
+      <c r="G5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{076DC3EE-449A-43DB-9031-C457E48E1447}">
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>66</v>
+      </c>
+      <c r="B1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>67</v>
+      </c>
+      <c r="B3" t="s">
+        <v>80</v>
+      </c>
+      <c r="C3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E3" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>67</v>
+      </c>
+      <c r="B4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D4" t="s">
+        <v>83</v>
+      </c>
+      <c r="E4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7FC4263-E33F-4DFE-9240-DD92FC1E7EF6}">
   <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -1102,7 +1340,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{29401365-B411-4B64-80A1-27BF962D067F}">
   <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>